<commit_message>
feat: add longitude latitude in import export proposal
</commit_message>
<xml_diff>
--- a/template-import.xlsx
+++ b/template-import.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29504"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Nyibuk\Project\ereses-api\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ndaru\Nyibuk\Project\e-api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C171EE5-638F-45E0-A476-49158EBB4104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F32EF7B-817D-4B1C-A2D9-FB98C2F2BD43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{FDDDA279-FAC0-4A70-B00C-FFCC8A12C05F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{FDDDA279-FAC0-4A70-B00C-FFCC8A12C05F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>No</t>
   </si>
@@ -109,6 +109,60 @@
   </si>
   <si>
     <t>Ini Deskripsi 8</t>
+  </si>
+  <si>
+    <t>Longitude</t>
+  </si>
+  <si>
+    <t>Latitude</t>
+  </si>
+  <si>
+    <t>105.2620</t>
+  </si>
+  <si>
+    <t>105.2621</t>
+  </si>
+  <si>
+    <t>105.2622</t>
+  </si>
+  <si>
+    <t>105.2623</t>
+  </si>
+  <si>
+    <t>105.2624</t>
+  </si>
+  <si>
+    <t>105.2625</t>
+  </si>
+  <si>
+    <t>105.2626</t>
+  </si>
+  <si>
+    <t>105.2627</t>
+  </si>
+  <si>
+    <t>-5.4297</t>
+  </si>
+  <si>
+    <t>-5.4298</t>
+  </si>
+  <si>
+    <t>-5.4299</t>
+  </si>
+  <si>
+    <t>-5.4300</t>
+  </si>
+  <si>
+    <t>-5.4301</t>
+  </si>
+  <si>
+    <t>-5.4302</t>
+  </si>
+  <si>
+    <t>-5.4303</t>
+  </si>
+  <si>
+    <t>-5.4304</t>
   </si>
 </sst>
 </file>
@@ -171,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -180,6 +234,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -200,9 +257,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -240,7 +297,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -346,7 +403,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -488,7 +545,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -496,17 +553,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AF7C223-C7C8-478D-9E20-C01B052A1BF4}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.85546875" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="30.42578125" customWidth="1"/>
-    <col min="4" max="4" width="41.7109375" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6.88671875" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="30.44140625" customWidth="1"/>
+    <col min="4" max="4" width="41.6640625" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -519,8 +577,14 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -533,8 +597,14 @@
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -547,8 +617,14 @@
       <c r="D3" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -561,8 +637,14 @@
       <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -575,8 +657,14 @@
       <c r="D5" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -589,8 +677,14 @@
       <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -603,8 +697,14 @@
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -617,8 +717,14 @@
       <c r="D8" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -631,8 +737,14 @@
       <c r="D9" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>

</xml_diff>